<commit_message>
Atualizar relatório com dados revisados
</commit_message>
<xml_diff>
--- a/data/CAP_Semana_2 DE MAIO.xlsx
+++ b/data/CAP_Semana_2 DE MAIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabriel\Desktop\Relatório_Felipe\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{510E6142-ED38-4ABE-9034-D1CF8628B859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72BEB2FC-9914-45F3-9959-BAABF165D17A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="2130" windowWidth="20640" windowHeight="11040" xr2:uid="{8D2EDE68-77A0-48FE-A03B-A2F0182CE2F6}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="186">
   <si>
     <t>id</t>
   </si>
@@ -272,9 +272,6 @@
   </si>
   <si>
     <t>FELIPE BALAGUER</t>
-  </si>
-  <si>
-    <t>02/05/2026 - PRORROGADO</t>
   </si>
   <si>
     <t>34191.12184 37858.002936 80685.880009 3 14340009616644</t>
@@ -1058,15 +1055,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="3" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1079,16 +1076,16 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="3" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="3" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1098,12 +1095,12 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="3" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="3" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1116,16 +1113,16 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1138,20 +1135,20 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1598,8 +1595,8 @@
       <c r="B2" s="68">
         <v>46139</v>
       </c>
-      <c r="C2" s="69" t="s">
-        <v>77</v>
+      <c r="C2" s="86">
+        <v>46158</v>
       </c>
       <c r="D2" s="70"/>
       <c r="E2" s="71" t="s">
@@ -1633,10 +1630,10 @@
         <v>27</v>
       </c>
       <c r="O2" s="71" t="s">
+        <v>77</v>
+      </c>
+      <c r="P2" s="73" t="s">
         <v>78</v>
-      </c>
-      <c r="P2" s="73" t="s">
-        <v>79</v>
       </c>
       <c r="Q2" s="74"/>
       <c r="R2" s="75"/>
@@ -1678,8 +1675,8 @@
       <c r="B3" s="78">
         <v>46139</v>
       </c>
-      <c r="C3" s="79" t="s">
-        <v>77</v>
+      <c r="C3" s="86">
+        <v>46158</v>
       </c>
       <c r="D3" s="80"/>
       <c r="E3" s="81" t="s">
@@ -1713,10 +1710,10 @@
         <v>27</v>
       </c>
       <c r="O3" s="81" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P3" s="83" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q3" s="84"/>
       <c r="R3" s="75"/>
@@ -1794,7 +1791,7 @@
         <v>69</v>
       </c>
       <c r="P4" s="90" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q4" s="91"/>
       <c r="R4" s="92"/>
@@ -1872,7 +1869,7 @@
         <v>52</v>
       </c>
       <c r="P5" s="90" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q5" s="91"/>
       <c r="R5" s="92"/>
@@ -1950,7 +1947,7 @@
       </c>
       <c r="O6" s="87"/>
       <c r="P6" s="90" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q6" s="91"/>
       <c r="R6" s="92"/>
@@ -2000,7 +1997,7 @@
         <v>28</v>
       </c>
       <c r="F7" s="94" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G7" s="88" t="s">
         <v>18</v>
@@ -2027,10 +2024,10 @@
         <v>27</v>
       </c>
       <c r="O7" s="88" t="s">
+        <v>82</v>
+      </c>
+      <c r="P7" s="90" t="s">
         <v>83</v>
-      </c>
-      <c r="P7" s="90" t="s">
-        <v>84</v>
       </c>
       <c r="Q7" s="91"/>
       <c r="R7" s="92"/>
@@ -2077,7 +2074,7 @@
       </c>
       <c r="D8" s="87"/>
       <c r="E8" s="88" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F8" s="87"/>
       <c r="G8" s="88" t="s">
@@ -2153,16 +2150,16 @@
       </c>
       <c r="D9" s="97"/>
       <c r="E9" s="98" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F9" s="99">
         <v>120323</v>
       </c>
       <c r="G9" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H9" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I9" s="100">
         <v>3282.19</v>
@@ -2381,7 +2378,7 @@
       </c>
       <c r="D12" s="97"/>
       <c r="E12" s="98" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F12" s="99">
         <v>193506</v>
@@ -2488,7 +2485,7 @@
         <v>52</v>
       </c>
       <c r="P13" s="90" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="Q13" s="91"/>
       <c r="R13" s="92"/>
@@ -2566,7 +2563,7 @@
         <v>45</v>
       </c>
       <c r="P14" s="90" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Q14" s="91"/>
       <c r="R14" s="92"/>
@@ -2643,7 +2640,7 @@
         <v>27</v>
       </c>
       <c r="O15" s="88" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P15" s="91"/>
       <c r="Q15" s="91"/>
@@ -2694,7 +2691,7 @@
         <v>57</v>
       </c>
       <c r="F16" s="94" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G16" s="88" t="s">
         <v>18</v>
@@ -2721,7 +2718,7 @@
         <v>27</v>
       </c>
       <c r="O16" s="88" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P16" s="91"/>
       <c r="Q16" s="91"/>
@@ -2799,7 +2796,7 @@
         <v>27</v>
       </c>
       <c r="O17" s="88" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P17" s="91"/>
       <c r="Q17" s="91"/>
@@ -2850,7 +2847,7 @@
         <v>57</v>
       </c>
       <c r="F18" s="94" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G18" s="88" t="s">
         <v>18</v>
@@ -2877,7 +2874,7 @@
         <v>27</v>
       </c>
       <c r="O18" s="88" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P18" s="91"/>
       <c r="Q18" s="91"/>
@@ -2955,7 +2952,7 @@
         <v>27</v>
       </c>
       <c r="O19" s="88" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P19" s="91"/>
       <c r="Q19" s="91"/>
@@ -3006,7 +3003,7 @@
         <v>57</v>
       </c>
       <c r="F20" s="94" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G20" s="88" t="s">
         <v>18</v>
@@ -3033,7 +3030,7 @@
         <v>27</v>
       </c>
       <c r="O20" s="88" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="P20" s="91"/>
       <c r="Q20" s="91"/>
@@ -3081,7 +3078,7 @@
       </c>
       <c r="D21" s="97"/>
       <c r="E21" s="98" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F21" s="97"/>
       <c r="G21" s="98" t="s">
@@ -3110,7 +3107,7 @@
       </c>
       <c r="O21" s="97"/>
       <c r="P21" s="104" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q21" s="104" t="s">
         <v>31</v>
@@ -3159,14 +3156,14 @@
       </c>
       <c r="D22" s="97"/>
       <c r="E22" s="98" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F22" s="97"/>
       <c r="G22" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H22" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I22" s="100">
         <v>3304</v>
@@ -3233,7 +3230,7 @@
       </c>
       <c r="D23" s="97"/>
       <c r="E23" s="98" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F23" s="99">
         <v>23752</v>
@@ -3385,7 +3382,7 @@
       </c>
       <c r="D25" s="87"/>
       <c r="E25" s="88" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F25" s="94">
         <v>5841</v>
@@ -3415,10 +3412,10 @@
         <v>27</v>
       </c>
       <c r="O25" s="88" t="s">
+        <v>101</v>
+      </c>
+      <c r="P25" s="90" t="s">
         <v>102</v>
-      </c>
-      <c r="P25" s="90" t="s">
-        <v>103</v>
       </c>
       <c r="Q25" s="91"/>
       <c r="R25" s="92"/>
@@ -3465,7 +3462,7 @@
       </c>
       <c r="D26" s="87"/>
       <c r="E26" s="88" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F26" s="87"/>
       <c r="G26" s="88" t="s">
@@ -3481,7 +3478,7 @@
         <v>1</v>
       </c>
       <c r="K26" s="88" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L26" s="88" t="s">
         <v>26</v>
@@ -3493,7 +3490,7 @@
         <v>27</v>
       </c>
       <c r="O26" s="88" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="P26" s="91"/>
       <c r="Q26" s="91"/>
@@ -4256,7 +4253,7 @@
         <v>8971143886</v>
       </c>
       <c r="P36" s="90" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q36" s="91"/>
       <c r="R36" s="92"/>
@@ -4334,7 +4331,7 @@
         <v>8971143886</v>
       </c>
       <c r="P37" s="90" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Q37" s="91"/>
       <c r="R37" s="92"/>
@@ -4533,7 +4530,7 @@
       </c>
       <c r="D40" s="87"/>
       <c r="E40" s="88" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F40" s="87"/>
       <c r="G40" s="88" t="s">
@@ -4561,10 +4558,10 @@
         <v>27</v>
       </c>
       <c r="O40" s="88" t="s">
+        <v>109</v>
+      </c>
+      <c r="P40" s="90" t="s">
         <v>110</v>
-      </c>
-      <c r="P40" s="90" t="s">
-        <v>111</v>
       </c>
       <c r="Q40" s="90" t="s">
         <v>31</v>
@@ -4613,7 +4610,7 @@
       </c>
       <c r="D41" s="87"/>
       <c r="E41" s="88" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F41" s="87"/>
       <c r="G41" s="88" t="s">
@@ -4641,10 +4638,10 @@
         <v>27</v>
       </c>
       <c r="O41" s="88" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P41" s="90" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="Q41" s="90" t="s">
         <v>31</v>
@@ -4693,7 +4690,7 @@
       </c>
       <c r="D42" s="87"/>
       <c r="E42" s="88" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F42" s="87"/>
       <c r="G42" s="88" t="s">
@@ -4721,10 +4718,10 @@
         <v>27</v>
       </c>
       <c r="O42" s="88" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P42" s="90" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="Q42" s="90" t="s">
         <v>31</v>
@@ -4773,7 +4770,7 @@
       </c>
       <c r="D43" s="87"/>
       <c r="E43" s="88" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F43" s="87"/>
       <c r="G43" s="88" t="s">
@@ -4801,10 +4798,10 @@
         <v>27</v>
       </c>
       <c r="O43" s="88" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P43" s="90" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="Q43" s="90" t="s">
         <v>31</v>
@@ -4853,7 +4850,7 @@
       </c>
       <c r="D44" s="87"/>
       <c r="E44" s="88" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F44" s="87"/>
       <c r="G44" s="88" t="s">
@@ -4881,10 +4878,10 @@
         <v>27</v>
       </c>
       <c r="O44" s="88" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P44" s="90" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="Q44" s="90" t="s">
         <v>31</v>
@@ -4933,14 +4930,14 @@
       </c>
       <c r="D45" s="87"/>
       <c r="E45" s="88" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F45" s="87"/>
       <c r="G45" s="88" t="s">
         <v>29</v>
       </c>
       <c r="H45" s="88" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I45" s="89">
         <v>48000</v>
@@ -4949,7 +4946,7 @@
         <v>1</v>
       </c>
       <c r="K45" s="88" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="L45" s="88" t="s">
         <v>21</v>
@@ -5009,7 +5006,7 @@
       </c>
       <c r="D46" s="87"/>
       <c r="E46" s="88" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F46" s="87"/>
       <c r="G46" s="88" t="s">
@@ -5037,10 +5034,10 @@
         <v>27</v>
       </c>
       <c r="O46" s="88" t="s">
+        <v>123</v>
+      </c>
+      <c r="P46" s="90" t="s">
         <v>124</v>
-      </c>
-      <c r="P46" s="90" t="s">
-        <v>125</v>
       </c>
       <c r="Q46" s="90" t="s">
         <v>31</v>
@@ -5297,14 +5294,14 @@
       </c>
       <c r="D50" s="97"/>
       <c r="E50" s="98" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F50" s="97"/>
       <c r="G50" s="98" t="s">
         <v>37</v>
       </c>
       <c r="H50" s="98" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I50" s="100">
         <v>52489.59</v>
@@ -5313,7 +5310,7 @@
         <v>1</v>
       </c>
       <c r="K50" s="98" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="L50" s="98" t="s">
         <v>21</v>
@@ -5326,7 +5323,7 @@
       </c>
       <c r="O50" s="97"/>
       <c r="P50" s="104" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q50" s="104" t="s">
         <v>31</v>
@@ -5375,16 +5372,16 @@
       </c>
       <c r="D51" s="97"/>
       <c r="E51" s="98" t="s">
+        <v>129</v>
+      </c>
+      <c r="F51" s="99" t="s">
         <v>130</v>
-      </c>
-      <c r="F51" s="99" t="s">
-        <v>131</v>
       </c>
       <c r="G51" s="98" t="s">
         <v>18</v>
       </c>
       <c r="H51" s="98" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I51" s="100">
         <v>163.96</v>
@@ -5527,7 +5524,7 @@
       </c>
       <c r="D53" s="97"/>
       <c r="E53" s="98" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F53" s="99">
         <v>2381</v>
@@ -5603,7 +5600,7 @@
       </c>
       <c r="D54" s="97"/>
       <c r="E54" s="98" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F54" s="99">
         <v>61147</v>
@@ -5679,7 +5676,7 @@
       </c>
       <c r="D55" s="97"/>
       <c r="E55" s="98" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F55" s="99">
         <v>934170</v>
@@ -5831,7 +5828,7 @@
       </c>
       <c r="D57" s="97"/>
       <c r="E57" s="98" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F57" s="97"/>
       <c r="G57" s="98" t="s">
@@ -5905,7 +5902,7 @@
       </c>
       <c r="D58" s="97"/>
       <c r="E58" s="98" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F58" s="97"/>
       <c r="G58" s="98" t="s">
@@ -6008,7 +6005,7 @@
       </c>
       <c r="O59" s="87"/>
       <c r="P59" s="90" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="Q59" s="91"/>
       <c r="R59" s="92"/>
@@ -6055,14 +6052,14 @@
       </c>
       <c r="D60" s="87"/>
       <c r="E60" s="88" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F60" s="87"/>
       <c r="G60" s="88" t="s">
         <v>35</v>
       </c>
       <c r="H60" s="88" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I60" s="89">
         <v>540</v>
@@ -6131,14 +6128,14 @@
       </c>
       <c r="D61" s="87"/>
       <c r="E61" s="88" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F61" s="87"/>
       <c r="G61" s="88" t="s">
+        <v>140</v>
+      </c>
+      <c r="H61" s="88" t="s">
         <v>141</v>
-      </c>
-      <c r="H61" s="88" t="s">
-        <v>142</v>
       </c>
       <c r="I61" s="89">
         <v>18000</v>
@@ -6159,10 +6156,10 @@
         <v>27</v>
       </c>
       <c r="O61" s="88" t="s">
+        <v>142</v>
+      </c>
+      <c r="P61" s="90" t="s">
         <v>143</v>
-      </c>
-      <c r="P61" s="90" t="s">
-        <v>144</v>
       </c>
       <c r="Q61" s="91"/>
       <c r="R61" s="92"/>
@@ -6292,7 +6289,7 @@
         <v>52</v>
       </c>
       <c r="P63" s="90" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q63" s="91"/>
       <c r="R63" s="92"/>
@@ -6573,7 +6570,7 @@
       </c>
       <c r="D67" s="87"/>
       <c r="E67" s="88" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F67" s="87"/>
       <c r="G67" s="88" t="s">
@@ -6601,10 +6598,10 @@
         <v>27</v>
       </c>
       <c r="O67" s="88" t="s">
+        <v>146</v>
+      </c>
+      <c r="P67" s="90" t="s">
         <v>147</v>
-      </c>
-      <c r="P67" s="90" t="s">
-        <v>148</v>
       </c>
       <c r="Q67" s="90" t="s">
         <v>31</v>
@@ -6653,7 +6650,7 @@
       </c>
       <c r="D68" s="87"/>
       <c r="E68" s="88" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F68" s="87"/>
       <c r="G68" s="88" t="s">
@@ -6682,7 +6679,7 @@
       </c>
       <c r="O68" s="87"/>
       <c r="P68" s="110" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="Q68" s="90" t="s">
         <v>31</v>
@@ -6731,7 +6728,7 @@
       </c>
       <c r="D69" s="87"/>
       <c r="E69" s="88" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F69" s="87"/>
       <c r="G69" s="88" t="s">
@@ -6760,7 +6757,7 @@
       </c>
       <c r="O69" s="87"/>
       <c r="P69" s="90" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Q69" s="90" t="s">
         <v>31</v>
@@ -6809,7 +6806,7 @@
       </c>
       <c r="D70" s="87"/>
       <c r="E70" s="88" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F70" s="87"/>
       <c r="G70" s="88" t="s">
@@ -6885,7 +6882,7 @@
       </c>
       <c r="D71" s="87"/>
       <c r="E71" s="88" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F71" s="87"/>
       <c r="G71" s="88" t="s">
@@ -6914,7 +6911,7 @@
       </c>
       <c r="O71" s="87"/>
       <c r="P71" s="90" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="Q71" s="90" t="s">
         <v>31</v>
@@ -6963,14 +6960,14 @@
       </c>
       <c r="D72" s="97"/>
       <c r="E72" s="98" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F72" s="97"/>
       <c r="G72" s="98" t="s">
+        <v>155</v>
+      </c>
+      <c r="H72" s="98" t="s">
         <v>156</v>
-      </c>
-      <c r="H72" s="98" t="s">
-        <v>157</v>
       </c>
       <c r="I72" s="100">
         <v>96500</v>
@@ -7039,7 +7036,7 @@
       </c>
       <c r="D73" s="97"/>
       <c r="E73" s="98" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F73" s="99">
         <v>2495590</v>
@@ -7115,7 +7112,7 @@
       </c>
       <c r="D74" s="97"/>
       <c r="E74" s="98" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F74" s="99">
         <v>36535</v>
@@ -8027,16 +8024,16 @@
       </c>
       <c r="D86" s="97"/>
       <c r="E86" s="98" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F86" s="99">
         <v>120767</v>
       </c>
       <c r="G86" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H86" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I86" s="100">
         <v>244.8</v>
@@ -8210,7 +8207,7 @@
       </c>
       <c r="O88" s="97"/>
       <c r="P88" s="104" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q88" s="101"/>
       <c r="R88" s="102"/>
@@ -8288,7 +8285,7 @@
       </c>
       <c r="O89" s="87"/>
       <c r="P89" s="90" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q89" s="91"/>
       <c r="R89" s="92"/>
@@ -8366,7 +8363,7 @@
       </c>
       <c r="O90" s="87"/>
       <c r="P90" s="90" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q90" s="91"/>
       <c r="R90" s="92"/>
@@ -8444,7 +8441,7 @@
       </c>
       <c r="O91" s="87"/>
       <c r="P91" s="90" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q91" s="91"/>
       <c r="R91" s="92"/>
@@ -8494,7 +8491,7 @@
         <v>28</v>
       </c>
       <c r="F92" s="94" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G92" s="88" t="s">
         <v>18</v>
@@ -8521,10 +8518,10 @@
         <v>27</v>
       </c>
       <c r="O92" s="88" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="P92" s="90" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q92" s="91"/>
       <c r="R92" s="92"/>
@@ -8571,7 +8568,7 @@
       </c>
       <c r="D93" s="87"/>
       <c r="E93" s="88" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F93" s="87"/>
       <c r="G93" s="88" t="s">
@@ -8647,7 +8644,7 @@
       </c>
       <c r="D94" s="87"/>
       <c r="E94" s="88" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F94" s="87"/>
       <c r="G94" s="88" t="s">
@@ -8676,7 +8673,7 @@
       </c>
       <c r="O94" s="87"/>
       <c r="P94" s="90" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Q94" s="90" t="s">
         <v>31</v>
@@ -8777,7 +8774,7 @@
       </c>
       <c r="D96" s="87"/>
       <c r="E96" s="88" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F96" s="87"/>
       <c r="G96" s="88" t="s">
@@ -8793,7 +8790,7 @@
         <v>1</v>
       </c>
       <c r="K96" s="88" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L96" s="88" t="s">
         <v>26</v>
@@ -8805,7 +8802,7 @@
         <v>27</v>
       </c>
       <c r="O96" s="88" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P96" s="90">
         <v>79</v>
@@ -8855,7 +8852,7 @@
       </c>
       <c r="D97" s="87"/>
       <c r="E97" s="88" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F97" s="94">
         <v>5939</v>
@@ -8885,10 +8882,10 @@
         <v>27</v>
       </c>
       <c r="O97" s="88" t="s">
+        <v>166</v>
+      </c>
+      <c r="P97" s="90" t="s">
         <v>167</v>
-      </c>
-      <c r="P97" s="90" t="s">
-        <v>168</v>
       </c>
       <c r="Q97" s="91"/>
       <c r="R97" s="92"/>
@@ -8964,7 +8961,7 @@
       </c>
       <c r="O98" s="87"/>
       <c r="P98" s="90" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Q98" s="91"/>
       <c r="R98" s="92"/>
@@ -9011,7 +9008,7 @@
       </c>
       <c r="D99" s="87"/>
       <c r="E99" s="88" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F99" s="87"/>
       <c r="G99" s="88" t="s">
@@ -9039,7 +9036,7 @@
         <v>27</v>
       </c>
       <c r="O99" s="88" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="P99" s="91"/>
       <c r="Q99" s="91"/>
@@ -9087,7 +9084,7 @@
       </c>
       <c r="D100" s="87"/>
       <c r="E100" s="88" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F100" s="87"/>
       <c r="G100" s="88" t="s">
@@ -9115,7 +9112,7 @@
         <v>27</v>
       </c>
       <c r="O100" s="88" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="P100" s="91"/>
       <c r="Q100" s="91"/>
@@ -9194,7 +9191,7 @@
       </c>
       <c r="O101" s="97"/>
       <c r="P101" s="104" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="Q101" s="101"/>
       <c r="R101" s="102"/>
@@ -9241,14 +9238,14 @@
       </c>
       <c r="D102" s="97"/>
       <c r="E102" s="98" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F102" s="97"/>
       <c r="G102" s="98" t="s">
         <v>35</v>
       </c>
       <c r="H102" s="98" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I102" s="100">
         <v>260</v>
@@ -9270,7 +9267,7 @@
       </c>
       <c r="O102" s="97"/>
       <c r="P102" s="104" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Q102" s="104" t="s">
         <v>31</v>
@@ -9319,14 +9316,14 @@
       </c>
       <c r="D103" s="97"/>
       <c r="E103" s="98" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F103" s="97"/>
       <c r="G103" s="98" t="s">
         <v>35</v>
       </c>
       <c r="H103" s="98" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I103" s="100">
         <v>949</v>
@@ -9348,7 +9345,7 @@
       </c>
       <c r="O103" s="97"/>
       <c r="P103" s="104" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Q103" s="104" t="s">
         <v>31</v>
@@ -9397,14 +9394,14 @@
       </c>
       <c r="D104" s="97"/>
       <c r="E104" s="98" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F104" s="97"/>
       <c r="G104" s="98" t="s">
         <v>35</v>
       </c>
       <c r="H104" s="98" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I104" s="100">
         <v>6875</v>
@@ -9471,16 +9468,16 @@
       </c>
       <c r="D105" s="97"/>
       <c r="E105" s="98" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F105" s="99">
         <v>35033</v>
       </c>
       <c r="G105" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H105" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I105" s="100">
         <v>3342.1</v>
@@ -9547,7 +9544,7 @@
       </c>
       <c r="D106" s="97"/>
       <c r="E106" s="98" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F106" s="99">
         <v>6614</v>
@@ -9775,7 +9772,7 @@
       </c>
       <c r="D109" s="97"/>
       <c r="E109" s="98" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F109" s="99">
         <v>2540</v>
@@ -10283,16 +10280,16 @@
       </c>
       <c r="D116" s="97"/>
       <c r="E116" s="98" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F116" s="99">
         <v>120821</v>
       </c>
       <c r="G116" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H116" s="98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I116" s="100">
         <v>6057.35</v>
@@ -10666,7 +10663,7 @@
         <v>73</v>
       </c>
       <c r="F121" s="94" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G121" s="88" t="s">
         <v>18</v>
@@ -10770,7 +10767,7 @@
         <v>52</v>
       </c>
       <c r="P122" s="90" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Q122" s="91"/>
       <c r="R122" s="92"/>
@@ -11304,7 +11301,7 @@
         <v>45</v>
       </c>
       <c r="P129" s="90" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="Q129" s="91"/>
       <c r="R129" s="92"/>

</xml_diff>